<commit_message>
Novas materias e questões
</commit_message>
<xml_diff>
--- a/Simulados Faculdade.xlsx
+++ b/Simulados Faculdade.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Página1" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Página1" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="544">
   <si>
     <t>Matéria</t>
   </si>
@@ -606,13 +606,1368 @@
   <si>
     <t xml:space="preserve">Fazer um consenso entre os três Evangelhos sinóticos.
 </t>
+  </si>
+  <si>
+    <t>Como filho amado/único, Jesus encarna o verdadeiro Israel, na condição daquele que irá sofrer pelo povo, tal como um cordeiro pascal. Essa condição é indicada pela comparação de Jesus com o seguinte personagem da história de Israel:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Abraão</t>
+  </si>
+  <si>
+    <t>Isaque</t>
+  </si>
+  <si>
+    <t>Esaú</t>
+  </si>
+  <si>
+    <t>Ismael.</t>
+  </si>
+  <si>
+    <t>As marcas textuais do evangelho de Lucas revelam que as comunidades para as quais foi escrito eram predominantemente...
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Judaicas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gentílicas.
+</t>
+  </si>
+  <si>
+    <t>Cristãs antigas.</t>
+  </si>
+  <si>
+    <t>Israelitas.</t>
+  </si>
+  <si>
+    <t>Qual é a mensagem Central do Evangelho de Marcos?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jesus, o sucessor de João.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jesus é o Messias, Filho de Deus.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jesus, o Libertador.
+</t>
+  </si>
+  <si>
+    <t>Jesus, o Filho do homem.</t>
+  </si>
+  <si>
+    <t>A palavra parábola vem do grego parabole que significa, literalmente:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Comparação.</t>
+  </si>
+  <si>
+    <t>Lançar ao lado.</t>
+  </si>
+  <si>
+    <t>Enigma.</t>
+  </si>
+  <si>
+    <t>Provérbios.</t>
+  </si>
+  <si>
+    <t>Blasfemar contra o Espírito Santo que acompanhou o ministério de Jesus equivale a:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rejeitar a mensagem do evangelho.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Um ato contra o próprio reino satânico.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aceitar entrar no reino de Deus.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ser condenado diretamente e sem perdão ao inferno.
+</t>
+  </si>
+  <si>
+    <t>Qual evangelho sinótico é considerado o mais antigo?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Mateus.</t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Marcos.</t>
+  </si>
+  <si>
+    <t>João</t>
+  </si>
+  <si>
+    <t>Na linguagem mais comum em manuais de exegese e hermenêutica bíblica os gêneros textuais são nomeados de:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formas literárias.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planos de expressão.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criações estilísticas.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano de conteúdo.
+</t>
+  </si>
+  <si>
+    <t>Em Apocalipse 21:1-15, João expõe a visão do novo mundo baseado nas:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tradições veterotestamentárias.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na saciedade que põe fim a toda fome.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bem-aventuranças de Jesus.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinda do reino.
+</t>
+  </si>
+  <si>
+    <t>Sinóticos deriva de duas palavras gregas que, literalmente, significam:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Harmonia</t>
+  </si>
+  <si>
+    <t>Biografia</t>
+  </si>
+  <si>
+    <t>Unidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visão comum.
+</t>
+  </si>
+  <si>
+    <t>Por que os escribas de Jerusalém acusaram Jesus de ser possesso por Belzebu?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque ele fazia milagres.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque comparavam Jesus a um ladrão.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque ele expulsava os demônios.
+</t>
+  </si>
+  <si>
+    <t>Porque achavam que ele praticava exorcismo.</t>
+  </si>
+  <si>
+    <t>A relação mais amistosa de Jesus com a tradição bíblica israelita é acentuada no Evangelho de:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Mateus</t>
+  </si>
+  <si>
+    <t>Marcos</t>
+  </si>
+  <si>
+    <t>Qual é a primeira característica da identidade messiânica de Jesus?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foi ao deserto para ser tentado.
+</t>
+  </si>
+  <si>
+    <t>A escolha dos discípulos.</t>
+  </si>
+  <si>
+    <t>Sua fidelidade filial.</t>
+  </si>
+  <si>
+    <t>O batismo de Jesus.</t>
+  </si>
+  <si>
+    <t>Qual advérbio, típico do evangelho de Marcos, ressalta a dinamicidade dos eventos?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Perfeitamente</t>
+  </si>
+  <si>
+    <t>Certamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imediatamente.
+</t>
+  </si>
+  <si>
+    <t>Infelizmente.</t>
+  </si>
+  <si>
+    <t>Jesus caminha da Galileia ao Jordão, deste ao deserto, então, de volta à Galileia. O percurso geográfico de Jesus é o percurso marcado pela:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Solidariedade</t>
+  </si>
+  <si>
+    <t>Santidade</t>
+  </si>
+  <si>
+    <t>Impureza.</t>
+  </si>
+  <si>
+    <t>Desprezo</t>
+  </si>
+  <si>
+    <t>Qual é o primeiro ato solidário de Jesus com pessoas impuras e pecadoras que concretiza sua solidariedade com eles?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elege o novo Israel.
+</t>
+  </si>
+  <si>
+    <t>Derrota os inimigos do Pai.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ora e busca forças ao pai.
+</t>
+  </si>
+  <si>
+    <t>Batismo de Jesus.</t>
+  </si>
+  <si>
+    <t>Qual é o primeiro ato público relatado do ministério de Jesus?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A perícope do chamado.</t>
+  </si>
+  <si>
+    <t>Tentação de Jesus.</t>
+  </si>
+  <si>
+    <t>O batismo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pregação do reino de Deus.
+</t>
+  </si>
+  <si>
+    <t>A mensagem central do Evangelho de Lucas: Jesus é o Messias, Filho do Homem e Filho de Deus, é similar aos seguintes evangelhos:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Mateus e João.</t>
+  </si>
+  <si>
+    <t>Marcos e João.</t>
+  </si>
+  <si>
+    <t>Tomé e Mateus.</t>
+  </si>
+  <si>
+    <t>Marcos e Mateus.</t>
+  </si>
+  <si>
+    <t>Para quem era essencial a exigência da lei?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Jesus</t>
+  </si>
+  <si>
+    <t>Fariseus</t>
+  </si>
+  <si>
+    <t>Palestinos</t>
+  </si>
+  <si>
+    <t>Deus</t>
+  </si>
+  <si>
+    <t>O evangelho de Marcos provavelmente foi escrito nos primeiros anos da década de:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Qual é o maior dos evangelhos?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Lucas.</t>
+  </si>
+  <si>
+    <t>João.</t>
+  </si>
+  <si>
+    <t>A função que coloca em destaque o código linguístico é:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Metalinguagem.</t>
+  </si>
+  <si>
+    <t>Conativa.</t>
+  </si>
+  <si>
+    <t>Referencial</t>
+  </si>
+  <si>
+    <t>Fática</t>
+  </si>
+  <si>
+    <t>É um exemplo de oração coordena Sindética Aditiva, a seguinte oração:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Não só pulei como também corri.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nem pulei e nem dancei durante a festa.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comprei um quilo de banana e fui trabalhar.
+</t>
+  </si>
+  <si>
+    <t>Todas as alternativas estão corretas.</t>
+  </si>
+  <si>
+    <t>Na frase: “ No coração da floresta existe um grande amor escondido”. É certo afirmar que é um exemplo de:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metáfora.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metonímia.
+</t>
+  </si>
+  <si>
+    <t>Sinestesia</t>
+  </si>
+  <si>
+    <t>Não pode ser considerada uma comparação a seguinte frase:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O rio é a lágrima de um oceano.</t>
+  </si>
+  <si>
+    <t>O rio é tal qual a lágrima de um oceano.</t>
+  </si>
+  <si>
+    <t>O rio é como a lágrima de um oceano.</t>
+  </si>
+  <si>
+    <t>O rio é semelhante a lágrima de um oceano.</t>
+  </si>
+  <si>
+    <t>Marque a alternativa correta:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O adjetivo concorda em gênero com o substantivo a que se refere.</t>
+  </si>
+  <si>
+    <t>O adjetivo só concorda com o número a que se refere o substantivo.</t>
+  </si>
+  <si>
+    <t>O adjetivo só tem uma forma.</t>
+  </si>
+  <si>
+    <t>O adjetivo não sofre flexão de grau.</t>
+  </si>
+  <si>
+    <t>Artigo é palavra que antepomos ao substantivo para:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Determiná-lo, indicar seu gênero e número.</t>
+  </si>
+  <si>
+    <t>Indicar o tempo verbal.</t>
+  </si>
+  <si>
+    <t>Classificar os adjetivos.</t>
+  </si>
+  <si>
+    <t>Regulamentar o uso dos pronomes.</t>
+  </si>
+  <si>
+    <t>O verbo pode aparecer na voz ativa e passiva. Marque a frase em que ele aparece na voz passiva:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O carro foi roubado.</t>
+  </si>
+  <si>
+    <t>A obra foi feita por ela.</t>
+  </si>
+  <si>
+    <t>A menina cortou-se.</t>
+  </si>
+  <si>
+    <t>Esta função tem por objetivo colocar o receptor numa posição de destaque. É uma afirmação que cabe somente à função:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Poética.</t>
+  </si>
+  <si>
+    <t>Metalinguística.</t>
+  </si>
+  <si>
+    <t>Conativa</t>
+  </si>
+  <si>
+    <t>Assinale a frase em que há erro de regência verbal:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A nota precisa de referência.</t>
+  </si>
+  <si>
+    <t>O dono realizou o levantamento das necessidades da loja.</t>
+  </si>
+  <si>
+    <t>Os médicos assistiram o simpósio e acharam-no muito interessante.</t>
+  </si>
+  <si>
+    <t>É preciso que todos cumpram às diretrizes da escola.</t>
+  </si>
+  <si>
+    <t>No enunciado “Trata-se de uma notícia muito boa!” O artigo é:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Definido plural.</t>
+  </si>
+  <si>
+    <t>Indefinido singular.</t>
+  </si>
+  <si>
+    <t>Definido singular.</t>
+  </si>
+  <si>
+    <t>Indefinido plural.</t>
+  </si>
+  <si>
+    <t>Filosofia da Religião</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas não descreve adequadamente a noção de sagrado?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sagrado diz respeito a algo espiritual e não se refere às coisas materiais e mundanas.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sagrado é uma qualidade inerente à pessoa ou objeto sacralizado, o que significa que independe das pessoas ou situações.
+</t>
+  </si>
+  <si>
+    <t>O sagrado jamais se confunde com o profano, e isso significa que no mundo há coisas ou pessoas que são desde sempre sagradas e coisas ou pessoas que são desde sempre profanas.</t>
+  </si>
+  <si>
+    <t>Nenhuma das afirmativas descreve bem a noção de sagrado.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas expressa uma perspectiva metafísica da Teologia?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A Teologia é a guardião da são doutrina, o que significa que suas descrições da realidade e da pessoa de Deus precisam se ancorar na revelação divina para que tenha validade universal.</t>
+  </si>
+  <si>
+    <t>Deus é uma realidade que independe do modo como o compreendemos, e qualquer conhecimento que se construa sobre ele deve ser buscado a partir dessa realidade autônoma e não nas descrições humanas sobre ele.</t>
+  </si>
+  <si>
+    <t>Pode-se dizer que a Teologia é o estudo da pessoa de Deus e de suas relações para com os humanos, e isso significa que deve ser compreendida numa perspectiva universal, independente dos contextos interpretativos.</t>
+  </si>
+  <si>
+    <t>Todas as afirmativas expressam uma perspectiva metafísica da Teologia.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas expressa melhor o efeito que o sagrado nos provoca?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O sagrado sempre nos causa temor, pois é isso em relação ao qual mantemos certa distância.</t>
+  </si>
+  <si>
+    <t>O sagrado sempre suscita intimidade, pois é isso em relação ao qual nos sentimos atraídos.</t>
+  </si>
+  <si>
+    <t>O sagrado é ambíguo, porquanto ao mesmo tempo em que dele mantemos certa distância pelo temor que nos provoca, por ele também nos sentimos atraídos e somos seduzidos a certa intimidade.</t>
+  </si>
+  <si>
+    <t>Nenhuma das afirmativas acima descrevem o efeito que o sagrado nos provoca.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas caracteriza adequadamente o sagrado?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O sagrado não é uma qualidade inerente à pessoa ou objeto sacralizado, o que significa que depende do sujeito que o venera.</t>
+  </si>
+  <si>
+    <t>Todas as afirmativas caracterizam adequadamente o sagrado.</t>
+  </si>
+  <si>
+    <t>O sagrado pode se confundir com o profano, e isso significa que no mundo não há coisas ou pessoas que são desde sempre sagradas e coisas ou pessoas que são desde sempre profanas.</t>
+  </si>
+  <si>
+    <t>O sagrado é qualitativamente diferente do profano, e o que é sagrado para uns é profano para outros.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas descreve melhor a noção de sagrado?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O sagrado diz respeito a algo espiritual e não se refere às coisas materiais e mundanas.</t>
+  </si>
+  <si>
+    <t>O sagrado é uma qualidade inerente à pessoa ou objeto sacralizado, o que significa que independe das pessoas ou situações.</t>
+  </si>
+  <si>
+    <t>O sagrado é qualitativamente diferente do profano, mas não é uma qualidade inerente à pessoa ou objeto sacralizado, o que significa que depende do sujeito que o venera — o que é sagrado para uns é profano para outros.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes alternativas NÃO caracteriza o papel da teologia numa sociedade democrática?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A teologia deve contribuir positivamente para a participação efetiva e consciente de pessoas religiosas na democracia.</t>
+  </si>
+  <si>
+    <t>É importante que a teologia se apresente de forma plural, mas de modo que as suas diferentes vozes e perspectivas não sejam vistas como concorrentes, mas como parceiras de diálogo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A teologia precisa se apresentar como guardiã da democracia, defendendo-a dos fundamentalismos religiosos dos mais diversos tipos que ameaçam as sociedades contemporâneas.
+</t>
+  </si>
+  <si>
+    <t>A teologia deve se apresentar em sua unidade fundamental, de maneira que sua pluralidade de vozes ceda lugar a uma só voz (unidade), a fim de que possa afetar positivamente a sociedade democrática.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas expressa uma perspectiva pós-metafísica da Teologia?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Pode-se dizer que a Teologia é o estudo das descrições humanas sobre Deus e suas relações para com os humanos, e isso significa que deve ser compreendida numa perspectiva local, a partir dos contextos interpretativos.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas possibilita inferir que o autor de Eclesiastes dialoga criticamente com as filosofias (sabedorias) do mundo grego e também do mundo oriental mesopotâmico?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Os mesmos conteúdos tratados no livro de Eclesiastes também são objetos de reflexão filosófica pelo mundo grego e mesopotâmico nos tempos iniciais da dominação de Judá pelos helenistas.</t>
+  </si>
+  <si>
+    <t>Todas as alternativas são verdadeiras.</t>
+  </si>
+  <si>
+    <t>O conceito de nulidade reúne o discurso judaico do discurso filosófico pós-metafísico na medida em que propõe o fim do fundamentalismo, tanto religioso quanto filosófico.</t>
+  </si>
+  <si>
+    <t>Há uma lógica, filosófica ou teológica, que atravessa a lógica poética, a desloca, se sustenta nela, mas não corresponde ao seu projeto. Uma lógica eivada de contrapontos, tensões e contradições, que obrigam leitores de Eclesiastes a exercícios intelectuais desafiadores.</t>
+  </si>
+  <si>
+    <t>Como Rorty vê a tarefa da Filosofia da religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Discute a relação da filosofia com a religião sob a ótica da tradução. Para ele, nesse esforço dialogal, a prioridade deveria ser o delineamento dos espaços próprios das diferentes linguagens da religião e da ciência.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Filosofia da Religião deve, com o auxílio das ciências, investigar em que medida as religiões se alinham com a verdade, afinal, uma de suas tarefas consiste em se buscar essa verdade.
+</t>
+  </si>
+  <si>
+    <t>A Filosofia da Religião pressupõe que o valor das ideias resida em sua utilidade ou conveniência, e não em sua fidelidade a um ideal transcendente.</t>
+  </si>
+  <si>
+    <t>Nenhuma das alternativas disponíveis.</t>
+  </si>
+  <si>
+    <t>A abordagem filosófica sistemática da religião é um produto do pensamento moderno. Quanto a isso, qual das afirmativas abaixo não é verdadeira?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A antiguidade clássica não considerou o tema como um aspecto particular de investigação, numa perspectiva sistematizada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A antiguidade clássica, bem como o pensamento cristão medieval, também elaboraram reflexões concernentes ao tema da religião.
+</t>
+  </si>
+  <si>
+    <t>A antiguidade clássica, bem como o pensamento cristão medieval, não elaboraram reflexões concernentes ao tema da religião.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abordagem sistemática, torna-se importante e necessária em virtude do conflito instaurado entre o mundo moderno, cada vez mais interessado no processo de libertação do homem a partir da ótica iluminista, e as doutrinas e instituições religiosas derivadas da tradição judaico-cristãs.
+</t>
+  </si>
+  <si>
+    <t>Qual das seguintes alternativas corresponde a uma tarefa da teologia em tom pós-metafísico?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A partir do diálogo público, defender a sociedade — especialmente as vítimas do capitalismo voraz — da dominação sistêmica.</t>
+  </si>
+  <si>
+    <t>A partir do diálogo religioso intramuros, defender os interesses do cristianismo da dominação antirreligiosa.</t>
+  </si>
+  <si>
+    <t>Defender a sociedade dos interesses de grupos defensores do ateísmo ou de religiões não-cristãs que interferem nas decisões do Estado a favor do cristianismo.</t>
+  </si>
+  <si>
+    <t>Defender a fé dos ataques à fé cristã, normalmente realizados a partir de conceitos derivados da ciência ou  da filosofia.</t>
+  </si>
+  <si>
+    <t>Qual das afirmativas Não demonstra uma tarefa da filosofia na contemporaneidade?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Mediar hermeneuticamente entre diferentes linguagens e não recair na posição de substituta da religião.</t>
+  </si>
+  <si>
+    <t>Desenvolver a dimensão epistemológica do saber.</t>
+  </si>
+  <si>
+    <t>Apoiar o aperfeiçoamento da democracia.</t>
+  </si>
+  <si>
+    <t>Desenvolver a dimensão terapêutica da racionalidade.</t>
+  </si>
+  <si>
+    <t>Qual o papel da teologia em tom pós-metafísico, em sua vertente libertadora?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Defender os direitos das pessoas mais empobrecidas e vitimadas pela globalização geográfica e simbólica da ideologia do livre-mercado e sua profetiza, a tecnologia.</t>
+  </si>
+  <si>
+    <t>Lutar por uma compreensão teológica mais fundamentada da realidade da libertação espiritual proposta pelo cristianismo ao longo de sua história.</t>
+  </si>
+  <si>
+    <t>Auxiliar a prática pastoral, na medida em que esta se baseia no fato de que as pessoas estão cada vez mais como “ovelhas sem pastor” e, portanto, necessitam de libertação.</t>
+  </si>
+  <si>
+    <t>Qual o período da história em que a filosofia assumiu o papel normativo, outrora pertencente à teologia e às vertentes clássicas da filosofia?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Primeira parte da Modernidade.</t>
+  </si>
+  <si>
+    <t>Durante toda a Modernidade.</t>
+  </si>
+  <si>
+    <t>Na Pós-Modernidade.</t>
+  </si>
+  <si>
+    <t>Durante a Idade Média</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas NÃO expressa um dos três grandes momentos de conflitividade entre filosofia e religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Quando filósofos tiveram de disputar com sacerdotes e líderes religiosos o direito de dizer a verdadee o prestígio social proveniente desse direito.</t>
+  </si>
+  <si>
+    <t>Quando o Cristianismo se tornou a religião oficial do Império Romano e a Igreja assumiu o controle da produção do saber legítimo, resultando numa predominância da teologia sobre a filosofia.</t>
+  </si>
+  <si>
+    <t>A partir da Modernidade, em que os interesses teológicos na busca pela verdade predominaram sobre os interesses filosóficos.</t>
+  </si>
+  <si>
+    <t>A partir da Modernidade até nossos dias, com os movimentos de secularização da sociedade, e a paulatina ascensão da ciência sobre a filosofia e a teologia.</t>
+  </si>
+  <si>
+    <t>Como Habermas vê a tarefa da filosofia da religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Para ele, o valor das ideias reside em sua utilidade, ou conveniência, e não na sua fidelidade a um ideal transcendente.</t>
+  </si>
+  <si>
+    <t>A filosofia, em tom pós-metafísico, não pode mais desempenhar o papel de discurso fundacional, mas deve assumir o lugar de mediadora, intérprete entre diferentes formas do saber humano. A filosofia da religião deveria se esforçar, primeiro, para, em diálogo com as pessoas e comunidades de fé, traduzir conceitos religiosos em linguagem não-religiosa, aberta.</t>
+  </si>
+  <si>
+    <t>A filosofia da religião deve, com o auxílio das ciências, investigar em que medida as religiões se alinham com a verdade, afinal, uma de suas tarefas consiste em se buscar essa verdade.</t>
+  </si>
+  <si>
+    <t>Resgatar a boa tradição.</t>
+  </si>
+  <si>
+    <t>Qual dos seguintes paradoxos aproxima o livro de Eclesiastes da reflexão filosófica contemporânea?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Se queremos compreender o “céu”, precisamos compreender a “terra”.</t>
+  </si>
+  <si>
+    <t>Se queremos compreender a vida, precisamos nos encantar com a morte.</t>
+  </si>
+  <si>
+    <t>Se queremos compreender a alma, precisamos aceitar o corpo.</t>
+  </si>
+  <si>
+    <t>Se queremos compreender a libertação, precisamos compreender a dominação.</t>
+  </si>
+  <si>
+    <t>A antiguidade clássica, bem como o pensamento cristão medieval, também elaboraram reflexões concernentes ao tema da religião.</t>
+  </si>
+  <si>
+    <t>A antiguidade clássica também considerou o tema como um aspecto particular de investigação, numa perspectiva sistematizada.</t>
+  </si>
+  <si>
+    <t>Abordagem sistemática, torna-se importante e necessária em virtude do conflito instaurado entre o mundo moderno, cada vez mais interessado no processo de libertação do homem a partir da ótica iluminista, e as doutrinas e instituições religiosas derivadas da tradição judaico-cristãs.</t>
+  </si>
+  <si>
+    <t>Qual a diferença entre a abordagem filosófica da religião e a abordagem da Psicologia da Religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), o enfoque da Psicologia da Religião é mais descritivo, afinal, parte do pressuposto de que interpretar um fato religioso implica em se conhecê-lo.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), para a Psicologia da Religião a religião é uma forma fundamental de coesão social, ou seja, o fenômeno religioso mostra a realidade social e é essencialmente comunitário.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), para a Psicologia da Religião os fatos religiosos espelham a psique humana, o que significa dizer que sem o ser humano, não há experiência religiosa, afinal, o sentimento religioso é uma elaboração do eros básico do ser humano.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), a Psicologia da Religião estuda a intencionalidade dos fatos religiosos, os testemunhos do ser humano religioso e o que para ele significam tais fatos, o que significa que o interesse está no modo como esse fenômeno se manifesta e como é recebido por aqueles que são adeptos dessas instituições.</t>
+  </si>
+  <si>
+    <t>Qual a diferença entre a abordagem filosófica da religião e a abordagem da Sociologia da Religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), o enfoque da Sociologia da Religião é mais descritivo, afinal, parte do pressuposto de que interpretar um fato religioso implica em se conhecê-lo.
+</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), para a Sociologia da Religião a religião é uma forma fundamental de coesão social, ou seja, o fenômeno religioso mostra a realidade social e é essencialmente comunitário.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), para a Sociologia da Religião os fatos religiosos espelham a psique humana, o que significa dizer que sem o ser humano, não há experiência religiosa, afinal, o sentimento religioso é uma elaboração do eros básico do ser humano.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), a Sociologia da Religião estuda a intencionalidade dos fatos religiosos, os testemunhos do ser humano religioso e o que para ele significam tais fatos, o que significa que o interesse está no modo como esse fenômeno se manifesta e como é recebido por aqueles que são adeptos dessas instituições.</t>
+  </si>
+  <si>
+    <t>“Quando qualquer coisa da criação de Deus é usada de maneira que não possa ser oferecida a Deus como um culto e não possa ser um ato de justiça, o universo foi profanado, por que o universo foi instrumentalizado para qualquer outra coisa que não seja o culto devido ao seu Criador. Então, isso quer dizer que qualquer movimento que descaracterize o propósito da criação de todas as coisas é um movimento profano. E qualquer movimento que leve a criação ao seu propósito, que é prestar ao Criador o culto que lhe é devido, é um movimento sagrado” (Cf. http://bit.ly/2jYSYyQ).
+Considere o trecho de uma fala de Ariovaldo Ramos, acima descrita, e responda: qual das seguintes alternativas não reflete o que está sendo dito?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Todas as coisas devem ser sacralizadas a fim de que prestem testemunho de que Deus é o Criador de tudo.</t>
+  </si>
+  <si>
+    <t>Sagrado e profano são operações do olhar, o que significa que as mesmas coisas podem ser sagradas e profanas, dependendo de como sejam vistas por cada pessoa.</t>
+  </si>
+  <si>
+    <t>O profano é compreendido de maneira negativa, como aquilo que supostamente não é dedicado a Deus ou que sobrevive de forma a descaracterizar o propósito da criação, que é prestar culto ao seu Criador.</t>
+  </si>
+  <si>
+    <t>Nenhuma das alternativas anteriores.</t>
+  </si>
+  <si>
+    <t>Qual das seguintes alternativas NÃO consiste numa sociedade pós-secular?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Uma sociedade na qual o discurso religioso, tanto quanto o discurso secular, tenham legitimidade na “arena pública”.</t>
+  </si>
+  <si>
+    <t>Uma sociedade na qual a consciência pública espelha muito mais um juízo normativo que tem consequências para o contato político entre cidadãos não-crentes e crentes.</t>
+  </si>
+  <si>
+    <t>Uma sociedade na qual não se tenta convencer a sociedade a destruir as crenças e instituições religiosas, nem mesmo impedir pessoas e instituições religiosas de participarem nos debates políticos nacionais.</t>
+  </si>
+  <si>
+    <t>Uma sociedade que legitima o secularismo e rejeita o fundamentalismo, enquanto perspectiva fundacional e antidemocrática.</t>
+  </si>
+  <si>
+    <t>Qual a diferença entre a abordagem filosófica da religião e a abordagem da Fenomenologia da Religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), o enfoque da Fenomenologia  da Religião é mais descritivo, afinal, parte do pressuposto de que interpretar um fato religioso implica em se conhecê-lo.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), para a Fenomenologia  da Religião a religião é uma forma fundamental de coesão social, ou seja, o fenômeno religioso mostra a realidade social e é essencialmente comunitário.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), para a Fenomenologia  da Religião os fatos religiosos espelham a psique humana, o que significa dizer que sem o ser humano, não há experiência religiosa, afinal, o sentimento religioso é uma elaboração do eros básico do ser humano.</t>
+  </si>
+  <si>
+    <t>Enquanto a Filosofia se preocupa com o absoluto na condição de ser e de fundamento de toda a realidade (perspectiva de cunho mais metafísico) ou se preocupa com o ser numa uma perspectiva hermenêutico-antropológica (perspectiva de cunho mais pós-metafísico), a Fenomenologia  da Religião estuda a intencionalidade dos fatos religiosos, os testemunhos do ser humano religioso e o que para ele significam tais fatos, o que significa que o interesse está no modo como esse fenômeno se manifesta e como é recebido por aqueles que são adeptos dessas instituições.</t>
+  </si>
+  <si>
+    <t>Contribuir para a integração dos saberes em face dos perigos da fragmentação do conhecimento e da cisão entre as diferentes dimensões da razão.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defender a fé dos ataques à fé cristã, normalmente realizados a partir de conceitos derivados da ciência ou  da filosofia.
+</t>
+  </si>
+  <si>
+    <t>Qual das seguintes afirmativas expressa um dos três grandes momentos de conflitividade entre filosofia e religião?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Quando cientistas tiveram de disputar com filósofos e líderes religiosos o direito de dizer a verdade e o prestígio social proveniente desse direito.</t>
+  </si>
+  <si>
+    <t>A Idade Média, caracterizada pelos movimentos de secularização da sociedade, e a paulatina ascensão da ciência sobre a filosofia e a teologia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defender a sociedade dos interesses, por vezes míopes, de instituições religiosas que interferem inadequadamente na discussão dos limites da ciência.
+</t>
+  </si>
+  <si>
+    <t>Interpretar os novos movimentos à luz dos clássicos e afirmar seu caráter de mestra e rainha do saber.</t>
+  </si>
+  <si>
+    <t>Em que termos Gianni Vattimo concebe a verdade revelada nas Escrituras?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Como a verdade do dogma, fruto da tradição.</t>
+  </si>
+  <si>
+    <t>Como a verdade da teologia, fruto da reflexão crítica.</t>
+  </si>
+  <si>
+    <t>Como a verdade da ciência, fruto da observação.</t>
+  </si>
+  <si>
+    <t>Como a verdade do amor, da caridade, fruto de um chamado à prática.</t>
+  </si>
+  <si>
+    <t>Por que se pode dizer que o sagrado é ambíguo?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sagrado é ambíguo, porquanto ao mesmo tempo em que dele mantemos certa distância pelo temor que nos provoca, por ele também nos sentimos atraídos e somos seduzidos a certa intimidade.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sagrado é ambíguo, porquanto se trata de objetos ou coisas que sempre trazem ambiguidade para aqueles que procuram entendê-lo.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sagrado é ambíguo porque pode estar no altar tanto do cristão, do budista, do muçulmano ou de qualquer outra religião.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sagrando, na realidade, não é ambíguo.
+</t>
+  </si>
+  <si>
+    <t>Psicologia Geral</t>
+  </si>
+  <si>
+    <t>A importância de Emil Kraepelin para o estudo das psicopatologias deve-se a que?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>As doenças mentais podem ser definidas a partir de desordens psíquicas em relação ao comportamento convencionado como padrão.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que a esquizofrenia não é uma coisa só, mas sim uma síndrome que supõe uma fragmentação e desorganização do funcionamento psicológico.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foi ele o responsável pela descrição e classificação dos transtornos mentais.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todas as respostas estão corretas.
+</t>
+  </si>
+  <si>
+    <t>Kurt Schneider os indivíduos do tipo “psicopatas fanáticos” são os que mais apresentam conteúdos e elementos religiosos em seu comportamento. Ele os divide em dois grupos que são:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fanáticos revolucionários e individualistas.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fanático expansivos e discretos.
+</t>
+  </si>
+  <si>
+    <t>Fanáticos liberais e conservadores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fanáticos cultos e incultos.
+</t>
+  </si>
+  <si>
+    <t>São os precursores da psicologia moderna:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platão e Aristóteles.
+</t>
+  </si>
+  <si>
+    <t>Sócrates e Platão.</t>
+  </si>
+  <si>
+    <t>Aristóteles e Sócrates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nenhuma das respostas.
+</t>
+  </si>
+  <si>
+    <t>Psicopatologia pode ser entendida como:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A classificação dos transtornos mentais.
+</t>
+  </si>
+  <si>
+    <t>O estudo aplicado dos sintomas anormais demonstrados na vida do indivíduo.</t>
+  </si>
+  <si>
+    <t>Uma síndrome que aborda só um aspecto da saúde mental.</t>
+  </si>
+  <si>
+    <t>Todas as respostas estão incorretas.</t>
+  </si>
+  <si>
+    <t>Foi desenvolvida por Gerald Kleman e Myrna Weissmann nos anos 70:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Terapia Comportamental.</t>
+  </si>
+  <si>
+    <t>Terapia Cognitiva.</t>
+  </si>
+  <si>
+    <t>Terapia Familiar e de Casal.</t>
+  </si>
+  <si>
+    <t>Terapia interpessoal (TIP).</t>
+  </si>
+  <si>
+    <t>Foi quem criou os testes de inteligência estática, abrindo portas para os testes de QI do mundo moderno:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ivan Pavlov.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">John Watson.
+</t>
+  </si>
+  <si>
+    <t>Alfred Binet.</t>
+  </si>
+  <si>
+    <t>Stanley Hall.</t>
+  </si>
+  <si>
+    <t>A quantos anos aproximadamente a psicologia é entendida como ciência?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">130 anos.
+</t>
+  </si>
+  <si>
+    <t>90 anos.</t>
+  </si>
+  <si>
+    <t>100 anos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nenhuma das respostas.
+</t>
+  </si>
+  <si>
+    <t>É o conceito mais antigo da Psicologia:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mecanicista.
+</t>
+  </si>
+  <si>
+    <t>Organicista.</t>
+  </si>
+  <si>
+    <t>Estruturalista</t>
+  </si>
+  <si>
+    <t>Vitalista</t>
+  </si>
+  <si>
+    <t>Considerando o pensamento de Jung sobre o objetivo da religião é certo afirmar quer:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O objetivo maior da religião é  identificar-se com a psique universal.
+</t>
+  </si>
+  <si>
+    <t>O objetivo maior da religião é não submergindo a consciência num mar de esquecimento inconsciente.</t>
+  </si>
+  <si>
+    <t>O objetivo maior da religião é integrar a consciência pessoal, através de recursos supremos.</t>
+  </si>
+  <si>
+    <t>Todas as respostas estão corretas.</t>
+  </si>
+  <si>
+    <t>“Matéria e vida são da mesma essência e a análise dos elementos de um objeto animado ou inanimado nos leva à total explicação das manifestações do objeto.” Está frase deve ser associada a qual conceito:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conceito Mecanicista.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conceito Vitalista.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conceito Organicista.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nenhum dos Conceitos  Apontados.
+</t>
+  </si>
+  <si>
+    <t>Qual a importância da fala no método Psicanalítico adotado por Freud?
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>O que Freud observou é que no exercício da fala, os pacientes por vezes demonstravam inibição quanto a imagens e ideias que surgiam.</t>
+  </si>
+  <si>
+    <t>Facilita a indução a sonhos eróticos e de prazer.</t>
+  </si>
+  <si>
+    <t>É importante porque somente por meio da fala o paciente pode ser analisado.</t>
+  </si>
+  <si>
+    <t>Nenhuma das alternativas está correta.</t>
+  </si>
+  <si>
+    <t>Foi quem ampliou o conceito científico que envolvia questões de psiquiatria criminal, neuropatologia, hipnose, psicolopatologia do trabalho e psicose infantil como dementia precosíssima. Está se falando de:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Freud.</t>
+  </si>
+  <si>
+    <t>Pinel.</t>
+  </si>
+  <si>
+    <t>De Sanctis.</t>
+  </si>
+  <si>
+    <t>Jung.</t>
+  </si>
+  <si>
+    <t>Os primeiros passos na direção do pensamento sobre o que poderia ser o mundo psicológico é atribuído a:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Sócrates</t>
+  </si>
+  <si>
+    <t>Platão.</t>
+  </si>
+  <si>
+    <t>Aristóteles.</t>
+  </si>
+  <si>
+    <t>Agostinho.</t>
+  </si>
+  <si>
+    <t>Tem seu fundamento nas teorias psicanalíticas da personalidade a seguinte terapia dinâmica:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Psicoterapia de Apoio.</t>
+  </si>
+  <si>
+    <t>Psicoterapia de Grupo.</t>
+  </si>
+  <si>
+    <t>Terapia Interpessoal.</t>
+  </si>
+  <si>
+    <t>Terapia comportamental.</t>
+  </si>
+  <si>
+    <t>Os fundadores da chamada psicologia experimental foram:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Wilhem Wundt , Ernst H.Weber, Gustav T. Fechner.</t>
+  </si>
+  <si>
+    <t>Pinel, Skinner e Ana Freud.</t>
+  </si>
+  <si>
+    <t>Platão, Sócrates e Aristóteles.</t>
+  </si>
+  <si>
+    <t>Nenhuma das respostas.</t>
+  </si>
+  <si>
+    <t>São Tomas de Aquino é influenciado em seu pensamento sobre essência e existência  por:  
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Sócrates.</t>
+  </si>
+  <si>
+    <t>Arquimedes</t>
+  </si>
+  <si>
+    <t>É o local em que se encontram as pulsões de vida e de morte:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>ID.</t>
+  </si>
+  <si>
+    <t>Ego.</t>
+  </si>
+  <si>
+    <t>Pré-consciente.</t>
+  </si>
+  <si>
+    <t>Consciente</t>
+  </si>
+  <si>
+    <t>Psicoterapias de apoio é apenas a que:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Está voltada primordialmente para o tratamento da depressão.</t>
+  </si>
+  <si>
+    <t>Tem como base o aprendizado como forma de entendimento da gênese dos sintomas, a manutenção e eliminação dos mesmos.</t>
+  </si>
+  <si>
+    <t>A intervenção do terapeuta é direta, funcionando como suporte, um ego auxiliar, e seu trabalho é focado na realidade atual do paciente.</t>
+  </si>
+  <si>
+    <t>São os três conceitos primordiais da psicologia:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Mecanicista, Filosofia e Estruturalista.</t>
+  </si>
+  <si>
+    <t>Organicista, Mecanicista e Vitalista.</t>
+  </si>
+  <si>
+    <t>Sensacionalista, Estruturalista, Fundamentalista.</t>
+  </si>
+  <si>
+    <t>“Essa teoria ocupa-se do ser humano como um todo e admite que qualquer evento psicológico é resultante de vários fatores e influenciam na conduta do indivíduo”. Esta frase faz parte do conceito:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Teoria Mecanicista.</t>
+  </si>
+  <si>
+    <t>Teoria Vitalista.</t>
+  </si>
+  <si>
+    <t>Teoria Organicista.</t>
+  </si>
+  <si>
+    <t>Teoria Analítica.</t>
+  </si>
+  <si>
+    <t>História e Cultura Helenística</t>
+  </si>
+  <si>
+    <t>Os gregos consideram a mensagem da cruz como loucura (1 Cor 1,22). De fato, quem poderia culpá-los, pois ninguém antes deles conhecera tão grande desenvolvimento cultural. Eles buscavam a sabedoria que traria sucesso na política, nos tribunais, na filosofia, no comércio, numa vida autárquica e, especialmente, a aprovação ou admiração de seus respectivos pares. A perspectiva de vida baseada nesses valores considera a “mensagem da cruz” uma afronta, pois a sabedoria humana considera loucura tudo o que é contrário a este modelo de vida. A “palavra da cruz” é também desprezada, pois a pessoa que Paulo proclamava havia aceitado um tipo de sofrimento e morte que eram considerados desonra e vergonha. A proclamação da “palavra da cruz” aos que buscavam honra e estima significava, portanto, uma grande afronta. Além disso, a renúncia à autarquia e a confiança posta inteiramente na ação de um “outro” significava a negação de tudo o que os gregos consideravam como caminho para o sucesso.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) Os gregos buscavam a sabedoria que traria sucesso na política, nos tribunais, na filosofia, no comércio, numa vida autárquica e, especialmente, a aprovação ou admiração de seus respectivos pares.
+( II ) A perspectiva de vida baseada nesses valores não considera a “mensagem da cruz” uma afronta, pois a sabedoria humana vê esta mensagem como adequada a este modelo de vida.
+( III ) A “palavra da cruz” é desprezada, pois a pessoa que Paulo proclamava havia aceitado um tipo de sofrimento e morte que eram considerados desonra e vergonha.
+( IV ) A renúncia à autarquia e a confiança posta na ação de um “outro” não significava a negação de tudo o que os gregos consideravam como caminho para o sucesso.
+Está correto o que se afirma em:
+Escolha uma opção</t>
+  </si>
+  <si>
+    <t>I e III apenas.</t>
+  </si>
+  <si>
+    <t>I e II apenas.</t>
+  </si>
+  <si>
+    <t>I, II e IV apenas.</t>
+  </si>
+  <si>
+    <t>II e IV apenas.</t>
+  </si>
+  <si>
+    <t>Através do processo de helenização, a língua e a cultura gregas se difundiram por todo o mundo mediterrâneo, especialmente graças às cidades fundadas por Alexandre e seus sucessores. Nestas cidades a civilização grega era implantada e se difundia pelo território ao seu derredor. O Judaísmo e o cristianismo nascente não podem ser entendidos de forma isolada do padrão cultural e religioso helenístico, mas o helenismo não pode ser visto como uma rua de mão única. A língua e a cultura gregas foram também influenciadas pelas culturas afro-asiáticas dos povos conquistados (desenvolveu-se o grego coinê, a forma da língua grega usada pela maioria da população, bem como no Novo Testamento), expandiram-se as religiões salvíficas de mistério (sincretismo de cultos afro-asiáticos com cultos greco-romanos), o Judaísmo ficou conhecido e era praticado em toda a região graças à dispersão de judeus (o que facilitou a expansão do Cristianismo).
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) O processo de helenização possibilitou a difusão da língua e a cultura gregas se difundiram por todo o mundo mediterrâneo, especialmente graças às cidades fundadas por Alexandre e seus sucessores.
+( II ) O helenismo é uma rua de mão única.
+( III ) Com o helenismo desenvolveu-se o grego coinê, a forma da língua grega usada pela maioria da população, bem como no Novo Testamento.
+( IV ) A dispersão dos judeus não facilitou o conhecimento do Judaísmo e não ajudou na expansão do Cristianismo.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>I, II e III apenas.</t>
+  </si>
+  <si>
+    <t>Um dos nomes mais conhecidos do Judaísmo fora de Israel é o de Filo, da cidade de Alexandria, um judeu que escreveu várias obras em que apresentou o Judaísmo ao mundo helênico. Filo lê a Escritura alegoricamente, associando-lhe significados que previamente não lhe diziam respeito. Ele compara a relação entre o sentido literal e o alegórico com a que existe entre o corpo e a alma, e o fato de que a alegoria quer alcançar algo invisível e mais elevado implica que este sentido não pode ser imediatamente acessível aos leitores. O intérprete experiente pode penetrar até este sentido mais elevado que Deus queria preservar do leitor comum, que fica preso no conteúdo literal. Para Filo, aqueles que “com base em pequenos indícios, conseguem entender o invisível através do visível” estão em condições de captar o sentido mais profundo das Escrituras.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) Filo, da cidade de Alexandria, escreveu várias obras em que apresentou o Judaísmo ao mundo helênico.
+( II ) A leitura alegórica da Escritura permite a Filo associar-lhe significados que previamente não lhe diziam respeito.
+( III ) Filo compara a relação entre o sentido literal e o alegórico com a que existe entre o corpo e a alma.
+( IV ) A leitura alegórica de Filo não procura apresentar o invisível através do visível.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+I, II e III apenas.
+</t>
+  </si>
+  <si>
+    <t>O exercício do senhorio de Cristo é totalmente distinto. É um senhorio que não conquista, mas reconcilia; não gera uniformidade, mas unidade. É um senhorio sem estratégias, mas com relacionamentos. Um senhorio cujo poder é exercido pelo Deus que faz a paz mediante a morte do seu próprio Filho, e não a dos seus inimigos. Na tradição judaico-cristã, a paz (shalom) é a plena harmonia que Deus estabelece na sua criação, com destaque para a justiça social, econômica e política que é a harmonia aplicada à convivência humana. Para restaurar a harmonia rompida da criação, Deus entrega Seu Filho à morte reconciliadora em benefício da criação alienada do Pai. Ou, nas palavras do próprio crucificado: “o Filho do Homem não veio para ser servido, mas para servir, e dar a sua vida em resgate de muitos” (Mc 10,45).
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) O senhorio de Cristo não significa conquista, mas reconciliação; não gera uniformidade, mas unidade.
+( II ) No senhorio de Cristo o poder é exercido pelo Deus que faz a paz mediante a morte do seu próprio Filho, e não a dos seus inimigos.
+( III ) Na tradição judaico-cristã, a paz (shalom), a plena harmonia que Deus estabelece na sua criação, não envolve a justiça social, econômica e política.
+( IV ) Para restaurar a harmonia rompida da criação, Deus entrega Seu Filho à morte reconciliadora em benefício da criação alienada do Pai.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>A tecnologia de produção era precária, fortemente dependente da mão-de-obra, mas em comparação com períodos anteriores era mais adequada, na medida em que se usavam ferramentas de ferro (especialmente arados) que permitiam maior produtividade, de modo que se produzia suficientemente para a subsistência da população geral do Império. O problema maior era a distribuição desses produtos, de tal forma que os governantes romanos tinham um papel importante na distribuição do trigo como um dos meios de manter a tranquilidade nos seus domínios. Avanços mais significativos se deram na construção de estradas e aquedutos, bem como no desenvolvimento de formas mais seguras de navegação ao longo das diversas costas do Mediterrâneo. Tais avanços foram necessários em função de dois fatores principais: o comércio e a manutenção do controle militar (exércitos dependem de boas estradas para alcançar com rapidez regiões de guerra). Em parte isto nos ajuda a entender a importância do controle dos exércitos na tomada e manutenção do poder imperial. Também nos ajuda a entender a importância da pax romana (“paz romana”) como mecanismo ideológico de apoio para a manutenção da tranquilidade nos domínios imperiais.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) Embora a tecnologia de produção fosse precária, na medida em que se usavam ferramentas de ferro que permitiam maior produtividade, se produzia suficientemente para a subsistência da população geral do Império.
+( II ) A distribuição desses produtos era tranquila, não necessitando dos governantes romanos para a sua realização.
+( III ) Aconteceram avanços na construção de estradas e aquedutos e no desenvolvimento de formas mais seguras de navegação ao longo das diversas costas do Mediterrâneo.
+( IV ) A pax romana (“paz romana”) era um mecanismo ideológico de apoio para a manutenção da tranquilidade nos domínios imperiais.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>I, III e IV apenas.</t>
+  </si>
+  <si>
+    <t>O Cristianismo nasceu durante um período em que todo o mundo helenístico estava sob o domínio do Império Romano. O mundo helenístico se localizava no entorno do mar Mediterrâneo. A palavra “mediterrâneo” significa “entre terras”, e o Mar Mediterrâneo era chamado mare internum (latim). Do ponto de vista geográfico, o mundo mediterrâneo engloba três continentes: Europa, Ásia e África – o que acarreta uma grande diversidade cultural, étnica, política, econômica e religiosa. Não só o domínio imperial romano, mas, já antes dele, a conquista de partes significativas da Ásia e África por Alexandre, o Grande (séc. IV a.C.), produziu uma espécie de homogeneização cultural-religiosa através da difusão do helenismo.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) O Cristianismo nasceu durante um período em que todo o mundo helenístico estava sob o domínio do Império Romano.
+( II ) A palavra “mediterrâneo” significa “entre terras”, e o Mar Mediterrâneo era chamado mare internum.
+( III ) Do ponto de vista geográfico, o mundo mediterrâneo engloba os continentes: Europa, Ásia, África e América.
+( IV ) A conquista de partes significativas da Ásia e África por Alexandre, o Grande (séc. IV a.C.), não produziu uma espécie de homogeneização cultural-religiosa através da difusão do helenismo.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>Para os saduceus, a pureza consistia na ausência, ou baixa presença, de defeitos ou máculas de tipo ritual (a presença dessas máculas definia a impureza). Havia máculas provisórias, que podiam ser eliminadas mediante sacrifícios e lavagens cerimoniais, e máculas permanentes que não podiam ser eliminadas. O critério de definição da pureza vinha da Torá sacerdotal, e aplicava ao mundo humano regras similares aplicadas ao mundo não-humano. Pessoas cuja mácula não podia ser eliminada estavam definitivamente afastadas de Deus e não poderiam participar da salvação do povo de Deus. Pessoas cuja mácula poderia ser removida deveriam se submeter às instruções sacerdotais para alcançar a purificação. Pessoas sem mácula eram aquelas que cumpriam rigorosamente as exigências da Torá sacerdotal e desfrutariam plenamente da salvação na era messiânica. Para os fariseus, que não negavam as noções de pureza sacerdotal, os sintomas mais importantes da pureza ou impureza tinham a ver com o cumprimento da Torá moral – especialmente a guarda do sábado, a ausência de contato com animais e/ou pessoas impuras, e a prática da piedade pessoal – especialmente a esmola, a oração e o jejum. Além das marcas da pureza vinculadas à ação humana, os fariseus também classificavam as pessoas em escalas de pureza conforme a sua condição física e de saúde (de modo similar à classificação dos saduceus). Assim, pessoas portadoras de deficiências físicas permanentes eram consideradas impuras (cegas, surdas, mudas, paralíticas, etc.); enquanto certas doenças mantinham as pessoas em situação de impureza até a sua cura (doenças da pele, especialmente aquelas cuja cura era desconhecida, eram as mais evidentes doenças relativas à impureza). Tanto para fariseus quanto para saduceus, as mulheres, pelo simples fato de serem mulheres, já estavam em condição pior do que os homens no quesito da pureza.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) Para os saduceus, a pureza não envolvia defeitos ou máculas de tipo ritual (a presença dessas máculas definia a impureza).
+( II ) O critério de definição da pureza dos saduceus vinha da Torá sacerdotal, e aplicava ao mundo humano regras similares aplicadas ao mundo não-humano.
+( III ) Para os fariseus, os sintomas mais importantes da pureza ou impureza tinham a ver com o cumprimento da Torá moral: a guarda do sábado, a ausência de contato com animais e/ou pessoas impuras, a prática da piedade pessoal.
+( IV ) Para fariseus e saduceus as mulheres tinham o mesmo valor que os homens no quesito da pureza.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>II e III apenas.</t>
+  </si>
+  <si>
+    <t>O dito de Jesus sobre odres novos e remendos novos é fundamental para entender o discurso do seu movimento. Não é possível criar um novo mundo sem rompermos com as amarras do velho mundo. O discurso do movimento de Jesus era um discurso de tipo profético-apocalíptico. Da profecia vem a intensa crítica contra toda forma de injustiça e dominação. Da apocalíptica vem a intensa expectativa de uma transformação radical da realidade social. De ambas vem a confiante certeza em Deus como o Senhor da história, que encaminhará essa transformação em conformidade com Sua vontade libertadora. É por isso que o tema central da mensagem de Jesus é o Reino de Deus. Jesus não prega a si mesmo como rei, fala de si mesmo como servo, como filho, como aquele que foi enviado pelo Pai para anunciar e concretizar a iminente chegada do Reino. Se Deus reina, não pode imperar a injustiça, a violência, a opressão. Se Deus reina, rompidos estão os grilhões da Lei e ativa a salvação pela graça.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) O dito de Jesus sobre odres novos e remendos novos é fundamental para entender o discurso do seu movimento, mas é possível criar um mundo novo sem rompermos com as amarras do velho mundo.
+( II ) A profecia crítica apenas pecados individuais e hipocrisia religiosa.
+( III ) A apocalíptica contém uma intensa expectativa de uma transformação radical da realidade social.
+( IV ) Jesus fala de si mesmo como servo, como filho, como aquele que foi enviado pelo Pai para anunciar e concretizar a iminente chegada do Reino.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>III e IV apenas.</t>
+  </si>
+  <si>
+    <t>Os essênios têm um papel peculiar no universo discursivo judaico, pois se constituía como uma cunha de oposição radical dentro do campo discursivo do Judaísmo Oficial. Eles não podem ser classificados exclusivamente como um grupo de resistência na medida em que não se opõem às características dominantes do discurso oficial. São, sim, um grupo de oposição, uma vez que disputa a legitimidade da liderança sacerdotal, bem como a legitimidade da interpretação da Torá – deste modo, ameaçam tanto a estabilidade política dos saduceus quanto a liderança teológica dos fariseus. Sua interpretação da Torá era peculiar, com três grandes ênfases: (a) um dualismo angelológico e moral, com características de determinismo; (b) um messianismo apocalíptico e guerreiro radical, que alimentava sonhos de libertação total da dominação imperial; (c) uma espiritualidade radical de seguimento das normas comunitárias e de afastamento da vida cotidiana, com vistas à plena consagração à vontade soberana do Senhor.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) Os essênios não podem ser classificados como um grupo de resistência na medida em que não se opõem às características dominantes do discurso oficial judaico.
+( II ) Uma das características da sua interpretação da Torá era um dualismo angelológico e moral, com características de determinismo.
+( III ) Um messianismo apocalíptico e guerreiro radical, que alimentava sonhos de libertação total da dominação imperial, não fazia parte da interpretação da Torá pelos essênios.
+( IV ) Os essênios estavam perfeitamente integrados na social e cultural judaica.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
+  </si>
+  <si>
+    <t>“É sintomático e carregado de sentido que desde o início, das primeiras vezes em que a pax romana é mencionada, se fala do imperador como chefe militar. O altar da paz ao Imperador Augusto, construído no simbólico lugar do Campo de Marte, deus da guerra, na verdade dava sentido à história da violência calcada no sucesso do vencedor. Sobre ele, o holocausto que queimava a vítima totalmente e por inteiro, sublinhava o fato do preço da paz proclamada e celebrada: o sangue derramado. A pax romana, portanto, é paz querida politicamente pelo imperador e seus mais altos funcionários, e estabelecida e garantida militarmente pela intervenção das legiões. A guerra que leva à vitória forma o pressuposto do tempo feliz da paz, no qual o Imperador triunfa. E este tempo feliz continua a ser assegurado pelas legiões e suas armas. Esta paz que Roma traz é paz-de-vitória para os romanos; para os vencidos, paz de submissão. Em teoria uma relação de direito entre dois parceiros, a pax romana é na realidade uma ordem de dominação. Roma é o parceiro que, a partir de si mesmo, ordena a relação e propõe as condições que o não romano deve aceitar, confirmando sua submissão ao poderoso Império que o protegia contra os ataques de outros povos estrangeiros. Esta paz estabelecida e mantida, portanto, com meios militares, é acompanhada de rios de sangue e lágrimas de enormes dimensões. Na verdade, nesta época da história, o mundo conhecido tem paz porque “todo o orbe terrestre” é dominado por Roma.
+De acordo com essa declaração, avalie as seguintes afirmações:
+( I  ) O altar da paz ao Imperador Augusto era muito mais a história da violência calcada no sucesso do vencedor.
+( II ) A pax romana (“paz romana”) era desejada politicamente pelo imperador e seus mais altos funcionários, mas estabelecida e garantida militarmente pela intervenção das legiões.
+( III ) A pax romana (“paz romana”) era a realidade da ordem de dominação do mundo da época por Roma.
+( IV ) Os povos conquistados aceitavam amigavelmente as propostas da paz por Roma.
+Está correto o que se afirma em:
+Escolha uma opção:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -636,8 +1991,18 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF001A1E"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF8E662E"/>
+      <name val="Poppins"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -656,6 +2021,12 @@
         <bgColor rgb="FFE7F3F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCEFDC"/>
+        <bgColor rgb="FFFCEFDC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -663,7 +2034,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -689,7 +2060,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -746,6 +2123,10 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -990,7 +2371,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="18.0"/>
     <col customWidth="1" min="2" max="2" width="53.63"/>
-    <col customWidth="1" min="3" max="3" width="51.38"/>
+    <col customWidth="1" min="3" max="3" width="22.88"/>
     <col customWidth="1" min="4" max="4" width="46.0"/>
     <col customWidth="1" min="5" max="5" width="49.5"/>
     <col customWidth="1" min="6" max="6" width="29.88"/>
@@ -2341,13 +3722,27 @@
       <c r="Z32" s="5"/>
     </row>
     <row r="33">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
+      <c r="A33" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
@@ -2369,13 +3764,27 @@
       <c r="Z33" s="5"/>
     </row>
     <row r="34">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
+      <c r="A34" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
@@ -2397,13 +3806,27 @@
       <c r="Z34" s="5"/>
     </row>
     <row r="35">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
+      <c r="A35" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
@@ -2425,13 +3848,27 @@
       <c r="Z35" s="5"/>
     </row>
     <row r="36">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
+      <c r="A36" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
@@ -2453,13 +3890,27 @@
       <c r="Z36" s="5"/>
     </row>
     <row r="37">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
+      <c r="A37" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
@@ -2481,13 +3932,27 @@
       <c r="Z37" s="5"/>
     </row>
     <row r="38">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
+      <c r="A38" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
@@ -2509,13 +3974,27 @@
       <c r="Z38" s="5"/>
     </row>
     <row r="39">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
+      <c r="A39" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
@@ -2537,13 +4016,27 @@
       <c r="Z39" s="5"/>
     </row>
     <row r="40">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
+      <c r="A40" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
@@ -2565,13 +4058,27 @@
       <c r="Z40" s="5"/>
     </row>
     <row r="41">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
+      <c r="A41" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
@@ -2593,13 +4100,27 @@
       <c r="Z41" s="5"/>
     </row>
     <row r="42">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
+      <c r="A42" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
@@ -2621,13 +4142,27 @@
       <c r="Z42" s="5"/>
     </row>
     <row r="43">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
+      <c r="A43" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
@@ -2649,13 +4184,27 @@
       <c r="Z43" s="5"/>
     </row>
     <row r="44">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
+      <c r="A44" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
@@ -2677,13 +4226,27 @@
       <c r="Z44" s="5"/>
     </row>
     <row r="45">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
+      <c r="A45" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
@@ -2705,13 +4268,27 @@
       <c r="Z45" s="5"/>
     </row>
     <row r="46">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
+      <c r="A46" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
@@ -2733,13 +4310,27 @@
       <c r="Z46" s="5"/>
     </row>
     <row r="47">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
+      <c r="A47" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
@@ -2761,13 +4352,27 @@
       <c r="Z47" s="5"/>
     </row>
     <row r="48">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
+      <c r="A48" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
@@ -2789,13 +4394,27 @@
       <c r="Z48" s="5"/>
     </row>
     <row r="49">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
+      <c r="A49" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
@@ -2817,13 +4436,27 @@
       <c r="Z49" s="5"/>
     </row>
     <row r="50">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
+      <c r="A50" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
@@ -2845,13 +4478,27 @@
       <c r="Z50" s="5"/>
     </row>
     <row r="51">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
+      <c r="A51" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C51" s="6">
+        <v>80.0</v>
+      </c>
+      <c r="D51" s="6">
+        <v>90.0</v>
+      </c>
+      <c r="E51" s="6">
+        <v>50.0</v>
+      </c>
+      <c r="F51" s="6">
+        <v>70.0</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
@@ -2873,13 +4520,27 @@
       <c r="Z51" s="5"/>
     </row>
     <row r="52">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
+      <c r="A52" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
@@ -2901,13 +4562,27 @@
       <c r="Z52" s="5"/>
     </row>
     <row r="53">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
+      <c r="A53" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
@@ -2929,13 +4604,27 @@
       <c r="Z53" s="5"/>
     </row>
     <row r="54">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
+      <c r="A54" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H54" s="5"/>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
@@ -2957,13 +4646,27 @@
       <c r="Z54" s="5"/>
     </row>
     <row r="55">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
+      <c r="A55" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H55" s="5"/>
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
@@ -2985,13 +4688,27 @@
       <c r="Z55" s="5"/>
     </row>
     <row r="56">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
+      <c r="A56" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H56" s="5"/>
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
@@ -3013,13 +4730,27 @@
       <c r="Z56" s="5"/>
     </row>
     <row r="57">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
+      <c r="A57" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H57" s="5"/>
       <c r="I57" s="5"/>
       <c r="J57" s="5"/>
@@ -3041,13 +4772,27 @@
       <c r="Z57" s="5"/>
     </row>
     <row r="58">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
+      <c r="A58" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H58" s="5"/>
       <c r="I58" s="5"/>
       <c r="J58" s="5"/>
@@ -3069,13 +4814,27 @@
       <c r="Z58" s="5"/>
     </row>
     <row r="59">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
+      <c r="A59" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H59" s="5"/>
       <c r="I59" s="5"/>
       <c r="J59" s="5"/>
@@ -3097,13 +4856,27 @@
       <c r="Z59" s="5"/>
     </row>
     <row r="60">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
+      <c r="A60" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H60" s="5"/>
       <c r="I60" s="5"/>
       <c r="J60" s="5"/>
@@ -3125,13 +4898,27 @@
       <c r="Z60" s="5"/>
     </row>
     <row r="61">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
+      <c r="A61" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H61" s="5"/>
       <c r="I61" s="5"/>
       <c r="J61" s="5"/>
@@ -3153,13 +4940,27 @@
       <c r="Z61" s="5"/>
     </row>
     <row r="62">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
+      <c r="A62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="F62" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H62" s="5"/>
       <c r="I62" s="5"/>
       <c r="J62" s="5"/>
@@ -3181,13 +4982,27 @@
       <c r="Z62" s="5"/>
     </row>
     <row r="63">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
+      <c r="A63" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="F63" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H63" s="5"/>
       <c r="I63" s="5"/>
       <c r="J63" s="5"/>
@@ -3209,13 +5024,27 @@
       <c r="Z63" s="5"/>
     </row>
     <row r="64">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5"/>
-      <c r="G64" s="5"/>
+      <c r="A64" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H64" s="5"/>
       <c r="I64" s="5"/>
       <c r="J64" s="5"/>
@@ -3237,13 +5066,27 @@
       <c r="Z64" s="5"/>
     </row>
     <row r="65">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5"/>
+      <c r="A65" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H65" s="5"/>
       <c r="I65" s="5"/>
       <c r="J65" s="5"/>
@@ -3265,13 +5108,27 @@
       <c r="Z65" s="5"/>
     </row>
     <row r="66">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
-      <c r="G66" s="5"/>
+      <c r="A66" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H66" s="5"/>
       <c r="I66" s="5"/>
       <c r="J66" s="5"/>
@@ -3293,13 +5150,27 @@
       <c r="Z66" s="5"/>
     </row>
     <row r="67">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
+      <c r="A67" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H67" s="5"/>
       <c r="I67" s="5"/>
       <c r="J67" s="5"/>
@@ -3321,13 +5192,27 @@
       <c r="Z67" s="5"/>
     </row>
     <row r="68">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-      <c r="G68" s="5"/>
+      <c r="A68" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H68" s="5"/>
       <c r="I68" s="5"/>
       <c r="J68" s="5"/>
@@ -3349,13 +5234,27 @@
       <c r="Z68" s="5"/>
     </row>
     <row r="69">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
+      <c r="A69" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H69" s="5"/>
       <c r="I69" s="5"/>
       <c r="J69" s="5"/>
@@ -3377,13 +5276,27 @@
       <c r="Z69" s="5"/>
     </row>
     <row r="70">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
+      <c r="A70" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H70" s="5"/>
       <c r="I70" s="5"/>
       <c r="J70" s="5"/>
@@ -3405,13 +5318,27 @@
       <c r="Z70" s="5"/>
     </row>
     <row r="71">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
+      <c r="A71" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H71" s="5"/>
       <c r="I71" s="5"/>
       <c r="J71" s="5"/>
@@ -3433,13 +5360,27 @@
       <c r="Z71" s="5"/>
     </row>
     <row r="72">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
+      <c r="A72" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H72" s="5"/>
       <c r="I72" s="5"/>
       <c r="J72" s="5"/>
@@ -3461,13 +5402,27 @@
       <c r="Z72" s="5"/>
     </row>
     <row r="73">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
-      <c r="F73" s="5"/>
-      <c r="G73" s="5"/>
+      <c r="A73" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H73" s="5"/>
       <c r="I73" s="5"/>
       <c r="J73" s="5"/>
@@ -3489,13 +5444,27 @@
       <c r="Z73" s="5"/>
     </row>
     <row r="74">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
-      <c r="G74" s="5"/>
+      <c r="A74" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H74" s="5"/>
       <c r="I74" s="5"/>
       <c r="J74" s="5"/>
@@ -3517,13 +5486,27 @@
       <c r="Z74" s="5"/>
     </row>
     <row r="75">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
-      <c r="G75" s="5"/>
+      <c r="A75" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H75" s="5"/>
       <c r="I75" s="5"/>
       <c r="J75" s="5"/>
@@ -3545,13 +5528,27 @@
       <c r="Z75" s="5"/>
     </row>
     <row r="76">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
+      <c r="A76" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H76" s="5"/>
       <c r="I76" s="5"/>
       <c r="J76" s="5"/>
@@ -3573,13 +5570,27 @@
       <c r="Z76" s="5"/>
     </row>
     <row r="77">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="5"/>
-      <c r="F77" s="5"/>
-      <c r="G77" s="5"/>
+      <c r="A77" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H77" s="5"/>
       <c r="I77" s="5"/>
       <c r="J77" s="5"/>
@@ -3601,13 +5612,27 @@
       <c r="Z77" s="5"/>
     </row>
     <row r="78">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
-      <c r="G78" s="5"/>
+      <c r="A78" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H78" s="5"/>
       <c r="I78" s="5"/>
       <c r="J78" s="5"/>
@@ -3629,13 +5654,27 @@
       <c r="Z78" s="5"/>
     </row>
     <row r="79">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="5"/>
-      <c r="F79" s="5"/>
-      <c r="G79" s="5"/>
+      <c r="A79" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H79" s="5"/>
       <c r="I79" s="5"/>
       <c r="J79" s="5"/>
@@ -3657,13 +5696,27 @@
       <c r="Z79" s="5"/>
     </row>
     <row r="80">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-      <c r="G80" s="5"/>
+      <c r="A80" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="G80" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H80" s="5"/>
       <c r="I80" s="5"/>
       <c r="J80" s="5"/>
@@ -3685,13 +5738,27 @@
       <c r="Z80" s="5"/>
     </row>
     <row r="81">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-      <c r="G81" s="5"/>
+      <c r="A81" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="G81" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H81" s="5"/>
       <c r="I81" s="5"/>
       <c r="J81" s="5"/>
@@ -3713,13 +5780,27 @@
       <c r="Z81" s="5"/>
     </row>
     <row r="82">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5"/>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
-      <c r="G82" s="5"/>
+      <c r="A82" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H82" s="5"/>
       <c r="I82" s="5"/>
       <c r="J82" s="5"/>
@@ -3741,13 +5822,27 @@
       <c r="Z82" s="5"/>
     </row>
     <row r="83">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-      <c r="G83" s="5"/>
+      <c r="A83" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="G83" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H83" s="5"/>
       <c r="I83" s="5"/>
       <c r="J83" s="5"/>
@@ -3769,13 +5864,27 @@
       <c r="Z83" s="5"/>
     </row>
     <row r="84">
-      <c r="A84" s="5"/>
-      <c r="B84" s="5"/>
-      <c r="C84" s="5"/>
-      <c r="D84" s="5"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-      <c r="G84" s="5"/>
+      <c r="A84" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H84" s="5"/>
       <c r="I84" s="5"/>
       <c r="J84" s="5"/>
@@ -3797,13 +5906,27 @@
       <c r="Z84" s="5"/>
     </row>
     <row r="85">
-      <c r="A85" s="5"/>
-      <c r="B85" s="5"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
-      <c r="G85" s="5"/>
+      <c r="A85" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="D85" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H85" s="5"/>
       <c r="I85" s="5"/>
       <c r="J85" s="5"/>
@@ -3825,13 +5948,27 @@
       <c r="Z85" s="5"/>
     </row>
     <row r="86">
-      <c r="A86" s="5"/>
-      <c r="B86" s="5"/>
-      <c r="C86" s="5"/>
-      <c r="D86" s="5"/>
-      <c r="E86" s="5"/>
-      <c r="F86" s="5"/>
-      <c r="G86" s="5"/>
+      <c r="A86" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="F86" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="G86" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H86" s="5"/>
       <c r="I86" s="5"/>
       <c r="J86" s="5"/>
@@ -3853,13 +5990,27 @@
       <c r="Z86" s="5"/>
     </row>
     <row r="87">
-      <c r="A87" s="5"/>
-      <c r="B87" s="5"/>
-      <c r="C87" s="5"/>
-      <c r="D87" s="5"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="5"/>
+      <c r="A87" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H87" s="5"/>
       <c r="I87" s="5"/>
       <c r="J87" s="5"/>
@@ -3881,13 +6032,27 @@
       <c r="Z87" s="5"/>
     </row>
     <row r="88">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="5"/>
-      <c r="E88" s="5"/>
-      <c r="F88" s="5"/>
-      <c r="G88" s="5"/>
+      <c r="A88" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="G88" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H88" s="5"/>
       <c r="I88" s="5"/>
       <c r="J88" s="5"/>
@@ -3909,13 +6074,27 @@
       <c r="Z88" s="5"/>
     </row>
     <row r="89">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
-      <c r="C89" s="5"/>
-      <c r="D89" s="5"/>
-      <c r="E89" s="5"/>
-      <c r="F89" s="5"/>
-      <c r="G89" s="5"/>
+      <c r="A89" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H89" s="5"/>
       <c r="I89" s="5"/>
       <c r="J89" s="5"/>
@@ -3937,13 +6116,27 @@
       <c r="Z89" s="5"/>
     </row>
     <row r="90">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="5"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
-      <c r="G90" s="5"/>
+      <c r="A90" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H90" s="5"/>
       <c r="I90" s="5"/>
       <c r="J90" s="5"/>
@@ -3965,13 +6158,27 @@
       <c r="Z90" s="5"/>
     </row>
     <row r="91">
-      <c r="A91" s="5"/>
-      <c r="B91" s="5"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="5"/>
-      <c r="E91" s="5"/>
-      <c r="F91" s="5"/>
-      <c r="G91" s="5"/>
+      <c r="A91" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H91" s="5"/>
       <c r="I91" s="5"/>
       <c r="J91" s="5"/>
@@ -3993,13 +6200,27 @@
       <c r="Z91" s="5"/>
     </row>
     <row r="92">
-      <c r="A92" s="5"/>
-      <c r="B92" s="5"/>
-      <c r="C92" s="5"/>
-      <c r="D92" s="5"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="5"/>
-      <c r="G92" s="5"/>
+      <c r="A92" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H92" s="5"/>
       <c r="I92" s="5"/>
       <c r="J92" s="5"/>
@@ -4021,13 +6242,27 @@
       <c r="Z92" s="5"/>
     </row>
     <row r="93">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="5"/>
-      <c r="E93" s="5"/>
-      <c r="F93" s="5"/>
-      <c r="G93" s="5"/>
+      <c r="A93" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H93" s="5"/>
       <c r="I93" s="5"/>
       <c r="J93" s="5"/>
@@ -4049,13 +6284,27 @@
       <c r="Z93" s="5"/>
     </row>
     <row r="94">
-      <c r="A94" s="5"/>
-      <c r="B94" s="5"/>
-      <c r="C94" s="5"/>
-      <c r="D94" s="5"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
-      <c r="G94" s="5"/>
+      <c r="A94" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H94" s="5"/>
       <c r="I94" s="5"/>
       <c r="J94" s="5"/>
@@ -4077,13 +6326,27 @@
       <c r="Z94" s="5"/>
     </row>
     <row r="95">
-      <c r="A95" s="5"/>
-      <c r="B95" s="5"/>
-      <c r="C95" s="5"/>
-      <c r="D95" s="5"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="5"/>
-      <c r="G95" s="5"/>
+      <c r="A95" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H95" s="5"/>
       <c r="I95" s="5"/>
       <c r="J95" s="5"/>
@@ -4105,13 +6368,27 @@
       <c r="Z95" s="5"/>
     </row>
     <row r="96">
-      <c r="A96" s="5"/>
-      <c r="B96" s="5"/>
-      <c r="C96" s="5"/>
-      <c r="D96" s="5"/>
-      <c r="E96" s="5"/>
-      <c r="F96" s="5"/>
-      <c r="G96" s="5"/>
+      <c r="A96" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H96" s="5"/>
       <c r="I96" s="5"/>
       <c r="J96" s="5"/>
@@ -4133,13 +6410,27 @@
       <c r="Z96" s="5"/>
     </row>
     <row r="97">
-      <c r="A97" s="5"/>
-      <c r="B97" s="5"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="5"/>
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5"/>
+      <c r="A97" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H97" s="5"/>
       <c r="I97" s="5"/>
       <c r="J97" s="5"/>
@@ -4161,13 +6452,27 @@
       <c r="Z97" s="5"/>
     </row>
     <row r="98">
-      <c r="A98" s="5"/>
-      <c r="B98" s="5"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="5"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
-      <c r="G98" s="5"/>
+      <c r="A98" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="D98" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="E98" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="F98" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="G98" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H98" s="5"/>
       <c r="I98" s="5"/>
       <c r="J98" s="5"/>
@@ -4189,13 +6494,27 @@
       <c r="Z98" s="5"/>
     </row>
     <row r="99">
-      <c r="A99" s="5"/>
-      <c r="B99" s="5"/>
-      <c r="C99" s="5"/>
-      <c r="D99" s="5"/>
-      <c r="E99" s="5"/>
-      <c r="F99" s="5"/>
-      <c r="G99" s="5"/>
+      <c r="A99" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D99" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="F99" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="G99" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H99" s="5"/>
       <c r="I99" s="5"/>
       <c r="J99" s="5"/>
@@ -4217,13 +6536,27 @@
       <c r="Z99" s="5"/>
     </row>
     <row r="100">
-      <c r="A100" s="5"/>
-      <c r="B100" s="5"/>
-      <c r="C100" s="5"/>
-      <c r="D100" s="5"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="5"/>
-      <c r="G100" s="5"/>
+      <c r="A100" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="F100" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="G100" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H100" s="5"/>
       <c r="I100" s="5"/>
       <c r="J100" s="5"/>
@@ -4245,13 +6578,27 @@
       <c r="Z100" s="5"/>
     </row>
     <row r="101">
-      <c r="A101" s="5"/>
-      <c r="B101" s="5"/>
-      <c r="C101" s="5"/>
-      <c r="D101" s="5"/>
-      <c r="E101" s="5"/>
-      <c r="F101" s="5"/>
-      <c r="G101" s="5"/>
+      <c r="A101" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="H101" s="5"/>
       <c r="I101" s="5"/>
       <c r="J101" s="5"/>
@@ -4273,13 +6620,27 @@
       <c r="Z101" s="5"/>
     </row>
     <row r="102">
-      <c r="A102" s="5"/>
-      <c r="B102" s="5"/>
-      <c r="C102" s="5"/>
-      <c r="D102" s="5"/>
-      <c r="E102" s="5"/>
-      <c r="F102" s="5"/>
-      <c r="G102" s="5"/>
+      <c r="A102" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="D102" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="F102" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="G102" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H102" s="5"/>
       <c r="I102" s="5"/>
       <c r="J102" s="5"/>
@@ -4301,13 +6662,27 @@
       <c r="Z102" s="5"/>
     </row>
     <row r="103">
-      <c r="A103" s="5"/>
-      <c r="B103" s="5"/>
-      <c r="C103" s="5"/>
-      <c r="D103" s="5"/>
-      <c r="E103" s="5"/>
-      <c r="F103" s="5"/>
-      <c r="G103" s="5"/>
+      <c r="A103" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="F103" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="G103" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H103" s="5"/>
       <c r="I103" s="5"/>
       <c r="J103" s="5"/>
@@ -4329,13 +6704,27 @@
       <c r="Z103" s="5"/>
     </row>
     <row r="104">
-      <c r="A104" s="5"/>
-      <c r="B104" s="5"/>
-      <c r="C104" s="5"/>
-      <c r="D104" s="5"/>
-      <c r="E104" s="5"/>
-      <c r="F104" s="5"/>
-      <c r="G104" s="5"/>
+      <c r="A104" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="D104" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="F104" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="G104" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H104" s="5"/>
       <c r="I104" s="5"/>
       <c r="J104" s="5"/>
@@ -4357,13 +6746,27 @@
       <c r="Z104" s="5"/>
     </row>
     <row r="105">
-      <c r="A105" s="5"/>
-      <c r="B105" s="5"/>
-      <c r="C105" s="5"/>
-      <c r="D105" s="5"/>
-      <c r="E105" s="5"/>
-      <c r="F105" s="5"/>
-      <c r="G105" s="5"/>
+      <c r="A105" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="D105" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="F105" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="G105" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H105" s="5"/>
       <c r="I105" s="5"/>
       <c r="J105" s="5"/>
@@ -4385,13 +6788,27 @@
       <c r="Z105" s="5"/>
     </row>
     <row r="106">
-      <c r="A106" s="5"/>
-      <c r="B106" s="5"/>
-      <c r="C106" s="5"/>
-      <c r="D106" s="5"/>
-      <c r="E106" s="5"/>
-      <c r="F106" s="5"/>
-      <c r="G106" s="5"/>
+      <c r="A106" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="D106" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="F106" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="G106" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H106" s="5"/>
       <c r="I106" s="5"/>
       <c r="J106" s="5"/>
@@ -4413,13 +6830,27 @@
       <c r="Z106" s="5"/>
     </row>
     <row r="107">
-      <c r="A107" s="5"/>
-      <c r="B107" s="5"/>
-      <c r="C107" s="5"/>
-      <c r="D107" s="5"/>
-      <c r="E107" s="5"/>
-      <c r="F107" s="5"/>
-      <c r="G107" s="5"/>
+      <c r="A107" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="F107" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="G107" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H107" s="5"/>
       <c r="I107" s="5"/>
       <c r="J107" s="5"/>
@@ -4441,13 +6872,27 @@
       <c r="Z107" s="5"/>
     </row>
     <row r="108">
-      <c r="A108" s="5"/>
-      <c r="B108" s="5"/>
-      <c r="C108" s="5"/>
-      <c r="D108" s="5"/>
-      <c r="E108" s="5"/>
-      <c r="F108" s="5"/>
-      <c r="G108" s="5"/>
+      <c r="A108" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="D108" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="E108" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="F108" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="G108" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H108" s="5"/>
       <c r="I108" s="5"/>
       <c r="J108" s="5"/>
@@ -4469,13 +6914,27 @@
       <c r="Z108" s="5"/>
     </row>
     <row r="109">
-      <c r="A109" s="5"/>
-      <c r="B109" s="5"/>
-      <c r="C109" s="5"/>
-      <c r="D109" s="5"/>
-      <c r="E109" s="5"/>
-      <c r="F109" s="5"/>
-      <c r="G109" s="5"/>
+      <c r="A109" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="D109" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="E109" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="F109" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="G109" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H109" s="5"/>
       <c r="I109" s="5"/>
       <c r="J109" s="5"/>
@@ -4497,13 +6956,27 @@
       <c r="Z109" s="5"/>
     </row>
     <row r="110">
-      <c r="A110" s="5"/>
-      <c r="B110" s="5"/>
-      <c r="C110" s="5"/>
-      <c r="D110" s="5"/>
-      <c r="E110" s="5"/>
-      <c r="F110" s="5"/>
-      <c r="G110" s="5"/>
+      <c r="A110" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B110" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="D110" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="E110" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="F110" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="G110" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H110" s="5"/>
       <c r="I110" s="5"/>
       <c r="J110" s="5"/>
@@ -4525,13 +6998,27 @@
       <c r="Z110" s="5"/>
     </row>
     <row r="111">
-      <c r="A111" s="5"/>
-      <c r="B111" s="5"/>
-      <c r="C111" s="5"/>
-      <c r="D111" s="5"/>
-      <c r="E111" s="5"/>
-      <c r="F111" s="5"/>
-      <c r="G111" s="5"/>
+      <c r="A111" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="D111" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="E111" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="F111" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="G111" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H111" s="5"/>
       <c r="I111" s="5"/>
       <c r="J111" s="5"/>
@@ -4553,13 +7040,27 @@
       <c r="Z111" s="5"/>
     </row>
     <row r="112">
-      <c r="A112" s="5"/>
-      <c r="B112" s="5"/>
-      <c r="C112" s="5"/>
-      <c r="D112" s="5"/>
-      <c r="E112" s="5"/>
-      <c r="F112" s="5"/>
-      <c r="G112" s="5"/>
+      <c r="A112" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="D112" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="E112" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="F112" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="G112" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H112" s="5"/>
       <c r="I112" s="5"/>
       <c r="J112" s="5"/>
@@ -4581,13 +7082,27 @@
       <c r="Z112" s="5"/>
     </row>
     <row r="113">
-      <c r="A113" s="5"/>
-      <c r="B113" s="5"/>
-      <c r="C113" s="5"/>
-      <c r="D113" s="5"/>
-      <c r="E113" s="5"/>
-      <c r="F113" s="5"/>
-      <c r="G113" s="5"/>
+      <c r="A113" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="C113" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="D113" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E113" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F113" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G113" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H113" s="5"/>
       <c r="I113" s="5"/>
       <c r="J113" s="5"/>
@@ -4609,13 +7124,27 @@
       <c r="Z113" s="5"/>
     </row>
     <row r="114">
-      <c r="A114" s="5"/>
-      <c r="B114" s="5"/>
-      <c r="C114" s="5"/>
-      <c r="D114" s="5"/>
-      <c r="E114" s="5"/>
-      <c r="F114" s="5"/>
-      <c r="G114" s="5"/>
+      <c r="A114" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B114" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D114" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="E114" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F114" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G114" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H114" s="5"/>
       <c r="I114" s="5"/>
       <c r="J114" s="5"/>
@@ -4637,13 +7166,27 @@
       <c r="Z114" s="5"/>
     </row>
     <row r="115">
-      <c r="A115" s="5"/>
-      <c r="B115" s="5"/>
-      <c r="C115" s="5"/>
-      <c r="D115" s="5"/>
-      <c r="E115" s="5"/>
-      <c r="F115" s="5"/>
-      <c r="G115" s="5"/>
+      <c r="A115" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B115" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="C115" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="D115" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F115" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G115" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H115" s="5"/>
       <c r="I115" s="5"/>
       <c r="J115" s="5"/>
@@ -4665,13 +7208,27 @@
       <c r="Z115" s="5"/>
     </row>
     <row r="116">
-      <c r="A116" s="5"/>
-      <c r="B116" s="5"/>
-      <c r="C116" s="5"/>
-      <c r="D116" s="5"/>
-      <c r="E116" s="5"/>
-      <c r="F116" s="5"/>
-      <c r="G116" s="5"/>
+      <c r="A116" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B116" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C116" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D116" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F116" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G116" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H116" s="5"/>
       <c r="I116" s="5"/>
       <c r="J116" s="5"/>
@@ -4693,13 +7250,27 @@
       <c r="Z116" s="5"/>
     </row>
     <row r="117">
-      <c r="A117" s="5"/>
-      <c r="B117" s="5"/>
-      <c r="C117" s="5"/>
-      <c r="D117" s="5"/>
-      <c r="E117" s="5"/>
-      <c r="F117" s="5"/>
-      <c r="G117" s="5"/>
+      <c r="A117" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D117" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E117" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="F117" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G117" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H117" s="5"/>
       <c r="I117" s="5"/>
       <c r="J117" s="5"/>
@@ -4721,13 +7292,27 @@
       <c r="Z117" s="5"/>
     </row>
     <row r="118">
-      <c r="A118" s="5"/>
-      <c r="B118" s="5"/>
-      <c r="C118" s="5"/>
-      <c r="D118" s="5"/>
-      <c r="E118" s="5"/>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5"/>
+      <c r="A118" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D118" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E118" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F118" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G118" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H118" s="5"/>
       <c r="I118" s="5"/>
       <c r="J118" s="5"/>
@@ -4749,13 +7334,27 @@
       <c r="Z118" s="5"/>
     </row>
     <row r="119">
-      <c r="A119" s="5"/>
-      <c r="B119" s="5"/>
-      <c r="C119" s="5"/>
-      <c r="D119" s="5"/>
-      <c r="E119" s="5"/>
-      <c r="F119" s="5"/>
-      <c r="G119" s="5"/>
+      <c r="A119" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="D119" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E119" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F119" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G119" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H119" s="5"/>
       <c r="I119" s="5"/>
       <c r="J119" s="5"/>
@@ -4777,13 +7376,27 @@
       <c r="Z119" s="5"/>
     </row>
     <row r="120">
-      <c r="A120" s="5"/>
-      <c r="B120" s="5"/>
-      <c r="C120" s="5"/>
-      <c r="D120" s="5"/>
-      <c r="E120" s="5"/>
-      <c r="F120" s="5"/>
-      <c r="G120" s="5"/>
+      <c r="A120" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B120" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D120" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F120" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G120" s="6" t="s">
+        <v>3</v>
+      </c>
       <c r="H120" s="5"/>
       <c r="I120" s="5"/>
       <c r="J120" s="5"/>
@@ -4805,13 +7418,27 @@
       <c r="Z120" s="5"/>
     </row>
     <row r="121">
-      <c r="A121" s="5"/>
-      <c r="B121" s="5"/>
-      <c r="C121" s="5"/>
-      <c r="D121" s="5"/>
-      <c r="E121" s="5"/>
-      <c r="F121" s="5"/>
-      <c r="G121" s="5"/>
+      <c r="A121" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B121" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="C121" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D121" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G121" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="H121" s="5"/>
       <c r="I121" s="5"/>
       <c r="J121" s="5"/>
@@ -4833,13 +7460,27 @@
       <c r="Z121" s="5"/>
     </row>
     <row r="122">
-      <c r="A122" s="5"/>
-      <c r="B122" s="5"/>
-      <c r="C122" s="5"/>
-      <c r="D122" s="5"/>
-      <c r="E122" s="5"/>
-      <c r="F122" s="5"/>
-      <c r="G122" s="5"/>
+      <c r="A122" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B122" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="C122" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="D122" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="E122" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F122" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="G122" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="H122" s="5"/>
       <c r="I122" s="5"/>
       <c r="J122" s="5"/>

</xml_diff>